<commit_message>
feat: embed authentic CIL 2025-26 images, 3-page multimodal executive summarization, and AST math verification in report generators
</commit_message>
<xml_diff>
--- a/backend/static/reports/Ministry_of_Coal_Report_2026.xlsx
+++ b/backend/static/reports/Ministry_of_Coal_Report_2026.xlsx
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Report ID: REP-2026-2BC4  |  Generated: 2026-09-04 23:50:39</t>
+          <t>Report ID: REP-2026-B56D  |  Generated: 2026-09-05 01:11:41</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>131608.9</v>
+        <v>768.1900000000001</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -528,11 +528,11 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>136067.7</v>
+        <v>798.8</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>96.72%</t>
+          <t>96.17%</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>126491.21</v>
+        <v>753.5</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -551,11 +551,11 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>131608.9</v>
+        <v>768.1900000000001</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>96.11% (Offtake)</t>
+          <t>98.09% (Offtake)</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>0.9672310180887895</v>
+        <v>0.9616800200300452</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>-3.28% vs Target</t>
+          <t>-3.83% vs Target</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>18</v>
+        <v>295</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>18</v>
+        <v>295</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -743,39 +743,39 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Gevra Expansion Mine</t>
+          <t>Mahanadi Coalfields Ltd (MCL)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chhattisgarh</t>
+          <t>Odisha</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SECL</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Opencast</t>
+          <t>Opencast/UG</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15265.48</v>
+        <v>218.31</v>
       </c>
       <c r="G4" t="n">
-        <v>14890.2</v>
+        <v>213.5</v>
       </c>
       <c r="H4" t="n">
-        <v>15500</v>
+        <v>225</v>
       </c>
       <c r="I4" t="n">
-        <v>98.48999999999999</v>
+        <v>97.03</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>11.60%</t>
+          <t>28.42%</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kusmunda Colliery</t>
+          <t>South Eastern Coalfields Ltd (SECL)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -800,24 +800,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Opencast</t>
+          <t>Opencast/UG</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>13842.1</v>
+        <v>176.29</v>
       </c>
       <c r="G5" t="n">
-        <v>13210.5</v>
+        <v>172.8</v>
       </c>
       <c r="H5" t="n">
-        <v>14000</v>
+        <v>185</v>
       </c>
       <c r="I5" t="n">
-        <v>98.87</v>
+        <v>95.29000000000001</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>10.52%</t>
+          <t>22.95%</t>
         </is>
       </c>
     </row>
@@ -827,17 +827,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dipka Project</t>
+          <t>Northern Coalfields Ltd (NCL)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chhattisgarh</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SECL</t>
+          <t>NCL</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -846,20 +846,20 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>12190.5</v>
+        <v>140.5</v>
       </c>
       <c r="G6" t="n">
-        <v>11950</v>
+        <v>139.1</v>
       </c>
       <c r="H6" t="n">
-        <v>12500</v>
+        <v>145</v>
       </c>
       <c r="I6" t="n">
-        <v>97.52</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>9.26%</t>
+          <t>18.29%</t>
         </is>
       </c>
     </row>
@@ -869,39 +869,39 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bhubaneswari OCP</t>
+          <t>Central Coalfields Ltd (CCL)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Odisha</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>CCL</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Opencast</t>
+          <t>Opencast/UG</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>11450.2</v>
+        <v>82.26000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>10980.4</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>12000</v>
+        <v>86</v>
       </c>
       <c r="I7" t="n">
-        <v>95.42</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8.70%</t>
+          <t>10.71%</t>
         </is>
       </c>
     </row>
@@ -911,39 +911,39 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lakhanpur Mine</t>
+          <t>Western Coalfields Ltd (WCL)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Odisha</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>WCL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Opencast</t>
+          <t>Opencast/UG</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>10320</v>
+        <v>68.03</v>
       </c>
       <c r="G8" t="n">
-        <v>9890</v>
+        <v>66.8</v>
       </c>
       <c r="H8" t="n">
-        <v>10500</v>
+        <v>71</v>
       </c>
       <c r="I8" t="n">
-        <v>98.29000000000001</v>
+        <v>95.81999999999999</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>7.84%</t>
+          <t>8.86%</t>
         </is>
       </c>
     </row>
@@ -953,39 +953,39 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Belpahar OCP</t>
+          <t>Eastern Coalfields Ltd (ECL)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Odisha</t>
+          <t>West Bengal</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>ECL</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Opencast</t>
+          <t>Opencast/UG</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>9840.15</v>
+        <v>52.08</v>
       </c>
       <c r="G9" t="n">
-        <v>9410.200000000001</v>
+        <v>50.9</v>
       </c>
       <c r="H9" t="n">
-        <v>10000</v>
+        <v>55</v>
       </c>
       <c r="I9" t="n">
-        <v>98.40000000000001</v>
+        <v>94.69</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>7.48%</t>
+          <t>6.78%</t>
         </is>
       </c>
     </row>
@@ -995,39 +995,39 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jayant Colliery</t>
+          <t>Bharat Coking Coal Ltd (BCCL)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NCL</t>
+          <t>BCCL</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Opencast</t>
+          <t>Opencast/UG</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9410.799999999999</v>
+        <v>35.52</v>
       </c>
       <c r="G10" t="n">
-        <v>9020.1</v>
+        <v>34.8</v>
       </c>
       <c r="H10" t="n">
-        <v>9800</v>
+        <v>37</v>
       </c>
       <c r="I10" t="n">
-        <v>96.03</v>
+        <v>96</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>7.15%</t>
+          <t>4.62%</t>
         </is>
       </c>
     </row>
@@ -1037,17 +1037,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dudhichua Project</t>
+          <t>North Eastern Coalfields (NEC)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Assam</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NCL</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1056,20 +1056,20 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>8920.6</v>
+        <v>0.2</v>
       </c>
       <c r="G11" t="n">
-        <v>8550</v>
+        <v>0.2</v>
       </c>
       <c r="H11" t="n">
-        <v>9200</v>
+        <v>0.3</v>
       </c>
       <c r="I11" t="n">
-        <v>96.95999999999999</v>
+        <v>66.67</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>6.78%</t>
+          <t>0.03%</t>
         </is>
       </c>
     </row>
@@ -1079,17 +1079,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nigahi Mine</t>
+          <t>Gevra Mega Expansion (SECL)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Chhattisgarh</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NCL</t>
+          <t>SECL</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1098,20 +1098,20 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>8450.299999999999</v>
+        <v>59.2</v>
       </c>
       <c r="G12" t="n">
-        <v>8100.2</v>
+        <v>58.1</v>
       </c>
       <c r="H12" t="n">
-        <v>8700</v>
+        <v>60</v>
       </c>
       <c r="I12" t="n">
-        <v>97.13</v>
+        <v>98.67</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>6.42%</t>
+          <t>7.71%</t>
         </is>
       </c>
     </row>
@@ -1121,17 +1121,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Amlohri Colliery</t>
+          <t>Kusmunda OCP (SECL)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Chhattisgarh</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NCL</t>
+          <t>SECL</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1140,20 +1140,20 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>7980.4</v>
+        <v>50.1</v>
       </c>
       <c r="G13" t="n">
-        <v>7650</v>
+        <v>49.3</v>
       </c>
       <c r="H13" t="n">
-        <v>8200</v>
+        <v>52</v>
       </c>
       <c r="I13" t="n">
-        <v>97.31999999999999</v>
+        <v>96.34999999999999</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>6.06%</t>
+          <t>6.52%</t>
         </is>
       </c>
     </row>
@@ -1163,17 +1163,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Rajmahal OCP</t>
+          <t>Dipka Project (SECL)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Chhattisgarh</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>SECL</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1182,20 +1182,20 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>7120.5</v>
+        <v>40</v>
       </c>
       <c r="G14" t="n">
-        <v>6890.3</v>
+        <v>39.2</v>
       </c>
       <c r="H14" t="n">
-        <v>7500</v>
+        <v>42</v>
       </c>
       <c r="I14" t="n">
-        <v>94.94</v>
+        <v>95.23999999999999</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>5.41%</t>
+          <t>5.21%</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1205,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Piprawar Project</t>
+          <t>Bhubaneswari OCP (MCL)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Odisha</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CCL</t>
+          <t>MCL</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1224,20 +1224,20 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>6450.2</v>
+        <v>35</v>
       </c>
       <c r="G15" t="n">
-        <v>6100</v>
+        <v>34.2</v>
       </c>
       <c r="H15" t="n">
-        <v>6800</v>
+        <v>36</v>
       </c>
       <c r="I15" t="n">
-        <v>94.86</v>
+        <v>97.22</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>4.90%</t>
+          <t>4.56%</t>
         </is>
       </c>
     </row>
@@ -1247,17 +1247,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ashoka Colliery</t>
+          <t>Jayant Colliery (NCL)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CCL</t>
+          <t>NCL</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1266,20 +1266,20 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4980.1</v>
+        <v>25</v>
       </c>
       <c r="G16" t="n">
-        <v>4720.5</v>
+        <v>24.8</v>
       </c>
       <c r="H16" t="n">
-        <v>5200</v>
+        <v>26</v>
       </c>
       <c r="I16" t="n">
-        <v>95.77</v>
+        <v>96.15000000000001</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3.78%</t>
+          <t>3.25%</t>
         </is>
       </c>
     </row>
@@ -1289,39 +1289,39 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Kalyaneshwari UG</t>
+          <t>Nigahi Project (NCL)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BCCL</t>
+          <t>NCL</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Underground</t>
+          <t>Opencast</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1240.3</v>
+        <v>23.5</v>
       </c>
       <c r="G17" t="n">
-        <v>1190</v>
+        <v>23.1</v>
       </c>
       <c r="H17" t="n">
-        <v>1500</v>
+        <v>24.5</v>
       </c>
       <c r="I17" t="n">
-        <v>82.69</v>
+        <v>95.92</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>0.94%</t>
+          <t>3.06%</t>
         </is>
       </c>
     </row>
@@ -1331,39 +1331,39 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Moonidih Deep UG</t>
+          <t>Dudhichua Project (NCL)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BCCL</t>
+          <t>NCL</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Underground</t>
+          <t>Opencast</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1120.4</v>
+        <v>22</v>
       </c>
       <c r="G18" t="n">
-        <v>1080.2</v>
+        <v>21.6</v>
       </c>
       <c r="H18" t="n">
-        <v>1300</v>
+        <v>23</v>
       </c>
       <c r="I18" t="n">
-        <v>86.18000000000001</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0.85%</t>
+          <t>2.86%</t>
         </is>
       </c>
     </row>
@@ -1373,39 +1373,39 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jhanjra UG Project</t>
+          <t>Piprawar Project (CCL)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>West Bengal</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>CCL</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Underground</t>
+          <t>Opencast</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1050.2</v>
+        <v>14.5</v>
       </c>
       <c r="G19" t="n">
-        <v>990</v>
+        <v>14.1</v>
       </c>
       <c r="H19" t="n">
-        <v>1200</v>
+        <v>15</v>
       </c>
       <c r="I19" t="n">
-        <v>87.52</v>
+        <v>96.67</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>1.89%</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sonepur Bazari OCP</t>
+          <t>Rajmahal OCP (ECL)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>West Bengal</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1434,20 +1434,20 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1010.5</v>
+        <v>17.2</v>
       </c>
       <c r="G20" t="n">
-        <v>940</v>
+        <v>16.9</v>
       </c>
       <c r="H20" t="n">
-        <v>1100</v>
+        <v>18</v>
       </c>
       <c r="I20" t="n">
-        <v>91.86</v>
+        <v>95.56</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>0.77%</t>
+          <t>2.24%</t>
         </is>
       </c>
     </row>
@@ -1457,17 +1457,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Khottadih Underground</t>
+          <t>Moonidih Deep UG (BCCL)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>West Bengal</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>BCCL</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1476,20 +1476,20 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>966.17</v>
+        <v>2.8</v>
       </c>
       <c r="G21" t="n">
-        <v>928.61</v>
+        <v>2.7</v>
       </c>
       <c r="H21" t="n">
-        <v>1067.7</v>
+        <v>3.2</v>
       </c>
       <c r="I21" t="n">
-        <v>90.48999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>0.36%</t>
         </is>
       </c>
     </row>

</xml_diff>